<commit_message>
TC_11013,11014,11015,11016,11021,11022 - Changes done.
</commit_message>
<xml_diff>
--- a/TestData/DeluxeTestData.xlsx
+++ b/TestData/DeluxeTestData.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="96">
   <si>
     <t>TestCaseId</t>
   </si>
@@ -125,151 +125,172 @@
     <t>PresetSaleItem2</t>
   </si>
   <si>
+    <t>ExistNumber</t>
+  </si>
+  <si>
     <t>TC_11013</t>
   </si>
   <si>
     <t>Sale</t>
   </si>
   <si>
+    <t>5/13 ZENTRO PROD TEST</t>
+  </si>
+  <si>
+    <t>umesh</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>umeshtest@testingxperts.com</t>
+  </si>
+  <si>
+    <t>Card</t>
+  </si>
+  <si>
+    <t>4444</t>
+  </si>
+  <si>
+    <t>Master</t>
+  </si>
+  <si>
+    <t>Door</t>
+  </si>
+  <si>
+    <t>no tax</t>
+  </si>
+  <si>
+    <t>ShirtProduct</t>
+  </si>
+  <si>
+    <t>CA</t>
+  </si>
+  <si>
+    <t>ac</t>
+  </si>
+  <si>
+    <t>United States</t>
+  </si>
+  <si>
+    <t>US</t>
+  </si>
+  <si>
+    <t>TestBook</t>
+  </si>
+  <si>
+    <t>Dollar Discount</t>
+  </si>
+  <si>
+    <t>TC_11015</t>
+  </si>
+  <si>
+    <t>0005</t>
+  </si>
+  <si>
+    <t>Amex</t>
+  </si>
+  <si>
+    <t>CA - California</t>
+  </si>
+  <si>
+    <t>Rustic Rubber</t>
+  </si>
+  <si>
+    <t>MobilePhone</t>
+  </si>
+  <si>
+    <t>default tax rate</t>
+  </si>
+  <si>
+    <t>TC_11021</t>
+  </si>
+  <si>
+    <t>6/15 Zentro test for robert esa</t>
+  </si>
+  <si>
+    <t>Paper</t>
+  </si>
+  <si>
+    <t>customer</t>
+  </si>
+  <si>
+    <t>umeshkumar@gmail.com</t>
+  </si>
+  <si>
+    <t>ACH/EFT</t>
+  </si>
+  <si>
+    <t>7244</t>
+  </si>
+  <si>
+    <t>1/11 colony</t>
+  </si>
+  <si>
+    <t>TX</t>
+  </si>
+  <si>
+    <t>Blvd Founders</t>
+  </si>
+  <si>
+    <t>newdiscount</t>
+  </si>
+  <si>
+    <t>FruitProduct</t>
+  </si>
+  <si>
+    <t>TC_11037</t>
+  </si>
+  <si>
+    <t>QA FEE TEST</t>
+  </si>
+  <si>
+    <t>HenryRR@gmail.com</t>
+  </si>
+  <si>
+    <t>6011111111111117</t>
+  </si>
+  <si>
+    <t>discover</t>
+  </si>
+  <si>
+    <t>No Tax</t>
+  </si>
+  <si>
+    <t>TX - Texas</t>
+  </si>
+  <si>
+    <t>BuyDoor</t>
+  </si>
+  <si>
+    <t>Testing</t>
+  </si>
+  <si>
+    <t>TextBook</t>
+  </si>
+  <si>
+    <t>VAT</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>TC_11031</t>
+  </si>
+  <si>
+    <t>4012888888881881</t>
+  </si>
+  <si>
+    <t>visa</t>
+  </si>
+  <si>
+    <t>SemiAnnually</t>
+  </si>
+  <si>
     <t>ZENTRO PROD TEST</t>
   </si>
   <si>
-    <t>umesh</t>
-  </si>
-  <si>
-    <t>test</t>
-  </si>
-  <si>
-    <t>umeshtest@testingxperts.com</t>
-  </si>
-  <si>
-    <t>Card</t>
-  </si>
-  <si>
-    <t>4444</t>
-  </si>
-  <si>
-    <t>Master</t>
-  </si>
-  <si>
-    <t>Door</t>
-  </si>
-  <si>
-    <t>no tax</t>
-  </si>
-  <si>
-    <t>ShirtProduct</t>
-  </si>
-  <si>
-    <t>CA</t>
-  </si>
-  <si>
-    <t>ac</t>
-  </si>
-  <si>
-    <t>United States</t>
-  </si>
-  <si>
-    <t>US</t>
-  </si>
-  <si>
-    <t>TestBook</t>
-  </si>
-  <si>
-    <t>Dollar Discount</t>
-  </si>
-  <si>
-    <t>TC_11015</t>
-  </si>
-  <si>
-    <t>0005</t>
-  </si>
-  <si>
-    <t>Amex</t>
-  </si>
-  <si>
-    <t>Rustic Rubber</t>
-  </si>
-  <si>
-    <t>MobilePhone</t>
-  </si>
-  <si>
-    <t>default tax rate</t>
-  </si>
-  <si>
-    <t>TC_11021</t>
-  </si>
-  <si>
     <t>zentro test for robert esa</t>
-  </si>
-  <si>
-    <t>ACH/EFT</t>
-  </si>
-  <si>
-    <t>7244</t>
-  </si>
-  <si>
-    <t>1/11 colony</t>
-  </si>
-  <si>
-    <t>TX</t>
-  </si>
-  <si>
-    <t>Blvd Founders</t>
-  </si>
-  <si>
-    <t>newdiscount</t>
-  </si>
-  <si>
-    <t>FruitProduct</t>
-  </si>
-  <si>
-    <t>TC_11037</t>
-  </si>
-  <si>
-    <t>QA FEE TEST</t>
-  </si>
-  <si>
-    <t>HenryRR@gmail.com</t>
-  </si>
-  <si>
-    <t>6011111111111117</t>
-  </si>
-  <si>
-    <t>discover</t>
-  </si>
-  <si>
-    <t>No Tax</t>
-  </si>
-  <si>
-    <t>TX - Texas</t>
-  </si>
-  <si>
-    <t>BuyDoor</t>
-  </si>
-  <si>
-    <t>Testing</t>
-  </si>
-  <si>
-    <t>TextBook</t>
-  </si>
-  <si>
-    <t>VAT</t>
-  </si>
-  <si>
-    <t>Monthly</t>
-  </si>
-  <si>
-    <t>TC_11031</t>
-  </si>
-  <si>
-    <t>4012888888881881</t>
-  </si>
-  <si>
-    <t>visa</t>
-  </si>
-  <si>
-    <t>SemiAnnually</t>
   </si>
   <si>
     <t>TC_11032</t>
@@ -1222,7 +1243,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AJ6"/>
+  <dimension ref="A1:AK6"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="5"/>
   <cols>
     <col min="1" max="1" width="14.8545454545455" customWidth="1"/>
@@ -1233,7 +1254,7 @@
     <col min="11" max="11" width="18.8545454545455" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36">
+    <row r="1" spans="1:37">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1342,408 +1363,417 @@
       <c r="AJ1" t="s">
         <v>35</v>
       </c>
+      <c r="AK1" t="s">
+        <v>36</v>
+      </c>
     </row>
-    <row r="2" ht="16" spans="1:26">
+    <row r="2" ht="16" spans="1:37">
       <c r="A2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I2">
         <v>1222342342</v>
       </c>
       <c r="J2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="L2">
         <v>444</v>
       </c>
       <c r="M2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="O2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="P2">
         <v>5</v>
       </c>
       <c r="Q2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="R2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="U2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="V2">
         <v>87686</v>
       </c>
       <c r="W2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="X2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Y2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Z2" t="s">
-        <v>53</v>
+        <v>54</v>
+      </c>
+      <c r="AK2">
+        <v>1117</v>
       </c>
     </row>
-    <row r="3" ht="16" spans="1:31">
+    <row r="3" ht="16" spans="1:37">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I3">
         <v>1222342342</v>
       </c>
       <c r="J3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L3">
         <v>444</v>
       </c>
       <c r="M3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="O3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="P3">
         <v>5</v>
       </c>
       <c r="Q3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="R3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T3" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="U3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="V3">
         <v>87686</v>
       </c>
       <c r="W3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="X3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Y3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Z3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="AA3">
         <v>123456</v>
       </c>
       <c r="AB3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="AC3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="AD3">
         <v>5</v>
       </c>
       <c r="AE3" t="s">
-        <v>59</v>
+        <v>61</v>
+      </c>
+      <c r="AK3">
+        <v>1117</v>
       </c>
     </row>
     <row r="4" ht="16" spans="1:36">
       <c r="A4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D4" t="s">
-        <v>39</v>
+        <v>64</v>
       </c>
       <c r="F4" t="s">
-        <v>39</v>
+        <v>64</v>
       </c>
       <c r="G4" t="s">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>41</v>
+        <v>66</v>
       </c>
       <c r="I4">
-        <v>1222342342</v>
+        <v>1232342345</v>
       </c>
       <c r="J4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="M4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="N4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="R4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S4" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="T4" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="U4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="V4">
         <v>30606</v>
       </c>
       <c r="W4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="X4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Y4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Z4" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="AA4">
         <v>123456</v>
       </c>
       <c r="AJ4" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" ht="16" spans="1:35">
       <c r="A5" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="E5">
         <v>50</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="I5">
         <v>1231232345</v>
       </c>
       <c r="J5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="L5">
         <v>444</v>
       </c>
       <c r="M5" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="N5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O5">
         <v>5</v>
       </c>
       <c r="P5" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="Q5" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="R5" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="S5" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="T5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="U5">
         <v>30606</v>
       </c>
       <c r="V5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="W5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="X5" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="Y5" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="Z5">
         <v>12345</v>
       </c>
       <c r="AB5" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="AC5">
         <v>10</v>
       </c>
       <c r="AD5" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="AG5" t="b">
         <v>1</v>
       </c>
       <c r="AH5" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="AI5" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" ht="16" spans="1:34">
       <c r="A6" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="E6">
         <v>50</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="I6">
         <v>1231232345</v>
       </c>
       <c r="J6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="L6">
         <v>444</v>
       </c>
       <c r="M6" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="N6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O6">
         <v>20</v>
       </c>
       <c r="P6" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="Q6" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="R6" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="S6" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="T6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="U6">
         <v>30606</v>
       </c>
       <c r="V6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="W6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="X6" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="Y6" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="AG6" t="b">
         <v>1</v>
       </c>
       <c r="AH6" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -1871,242 +1901,242 @@
     </row>
     <row r="2" ht="16" spans="1:26">
       <c r="A2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="D2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I2">
         <v>1222342342</v>
       </c>
       <c r="J2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="L2">
         <v>444</v>
       </c>
       <c r="M2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="O2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="P2">
         <v>5</v>
       </c>
       <c r="Q2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="R2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="U2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="V2">
         <v>87686</v>
       </c>
       <c r="W2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="X2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Y2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Z2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" ht="16" spans="1:31">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="D3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I3">
         <v>1222342342</v>
       </c>
       <c r="J3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L3">
         <v>444</v>
       </c>
       <c r="M3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="O3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="P3">
         <v>5</v>
       </c>
       <c r="Q3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="R3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="U3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="V3">
         <v>87686</v>
       </c>
       <c r="W3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="X3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Y3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Z3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="AA3">
         <v>123456</v>
       </c>
       <c r="AB3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="AC3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="AD3">
         <v>5</v>
       </c>
       <c r="AE3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" ht="16" spans="1:36">
       <c r="A4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>61</v>
+        <v>91</v>
       </c>
       <c r="D4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I4">
         <v>1222342342</v>
       </c>
       <c r="J4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="M4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="N4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="R4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S4" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="T4" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="U4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="V4">
         <v>30606</v>
       </c>
       <c r="W4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="X4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Y4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Z4" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="AA4">
         <v>123456</v>
       </c>
       <c r="AJ4" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" ht="16" spans="8:11">
@@ -2115,245 +2145,243 @@
     </row>
     <row r="6" ht="16" spans="1:35">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="E6">
         <v>50</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="I6">
         <v>1231232345</v>
       </c>
       <c r="J6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="L6">
         <v>444</v>
       </c>
       <c r="M6" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="N6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O6">
         <v>5</v>
       </c>
       <c r="P6" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="Q6" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="R6" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="S6" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="T6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="U6">
         <v>30606</v>
       </c>
       <c r="V6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="W6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="X6" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="Y6" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="Z6">
         <v>12345</v>
       </c>
       <c r="AB6" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="AC6">
         <v>10</v>
       </c>
       <c r="AD6" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="AG6" t="b">
         <v>1</v>
       </c>
       <c r="AH6" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="AI6" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" ht="16" spans="1:34">
       <c r="A7" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C7" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="E7">
         <v>50</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="I7">
         <v>1231232345</v>
       </c>
       <c r="J7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="L7">
         <v>444</v>
       </c>
       <c r="M7" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="N7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O7">
         <v>20</v>
       </c>
       <c r="P7" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="Q7" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="R7" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="S7" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="T7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="U7">
         <v>30606</v>
       </c>
       <c r="V7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="W7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="X7" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="Y7" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="AG7" t="b">
         <v>1</v>
       </c>
       <c r="AH7" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" ht="16" spans="8:11">
       <c r="H10" s="1"/>
-      <c r="I10"/>
-      <c r="J10"/>
       <c r="K10" s="2"/>
     </row>
     <row r="11" ht="16" spans="1:32">
       <c r="A11" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="B11" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C11" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="E11">
         <v>50</v>
       </c>
       <c r="F11" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="G11" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="I11">
         <v>1231232345</v>
       </c>
       <c r="J11" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="L11">
         <v>444</v>
       </c>
       <c r="M11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O11">
         <v>50</v>
       </c>
       <c r="P11" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="Q11" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="R11" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="S11" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="T11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="U11">
         <v>30606</v>
       </c>
       <c r="V11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="W11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="X11" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="Y11" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="Z11">
         <v>12345</v>

</xml_diff>